<commit_message>
refactor: UI 业务逻辑收敛到 activity 包
- 新增 src/activity/recipient_bulk：收件人文件解析(excel/txt)+合并
- 新增 src/activity/mail_query：邮件查询逻辑
- MainGUI 收件人选择/合并/查询响应改为调用 activity 层
- 修复合并逻辑中分号无法正确拆分的去重 bug
- .gitignore 排除含真实凭据的本地测试目录
</commit_message>
<xml_diff>
--- a/ProjectDescription/FunctionNameReg.xlsx
+++ b/ProjectDescription/FunctionNameReg.xlsx
@@ -15,6 +15,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="main" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="path_manager" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="database" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="activity_recipient_bulk" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="activity_mail_query" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,13 +26,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -53,8 +58,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1709,6 +1715,114 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>函数名/类名</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>类型</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>参数</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>返回值</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>函数意义</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>位置</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>记录/修改时间</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>queryEmails</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>函数</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>db&lt;MailDatabase&gt;; category&lt;str|None&gt;; condition&lt;dict&gt;</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>list&lt;dict&gt;</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>按条件查询邮件(主题/收件人/发件人/日期范围)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>(src/activity/mail_query.py)[queryEmails:19]</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-08-23 20:51:33</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -2190,7 +2304,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I156"/>
+  <dimension ref="A1:I180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -7138,7 +7252,6 @@
         </is>
       </c>
     </row>
-    <row r="131"/>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
@@ -7477,7 +7590,6 @@
         </is>
       </c>
     </row>
-    <row r="141"/>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
@@ -7520,7 +7632,6 @@
         </is>
       </c>
     </row>
-    <row r="143"/>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
@@ -7563,7 +7674,6 @@
         </is>
       </c>
     </row>
-    <row r="145"/>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
@@ -7601,7 +7711,6 @@
         </is>
       </c>
     </row>
-    <row r="147"/>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
@@ -7644,7 +7753,6 @@
         </is>
       </c>
     </row>
-    <row r="149"/>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
@@ -7687,7 +7795,6 @@
         </is>
       </c>
     </row>
-    <row r="151"/>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
@@ -7730,7 +7837,6 @@
         </is>
       </c>
     </row>
-    <row r="153"/>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
@@ -7773,7 +7879,6 @@
         </is>
       </c>
     </row>
-    <row r="155"/>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
@@ -7813,6 +7918,505 @@
       <c r="H156" t="inlineStr">
         <is>
           <t>新增(替代旧占位)</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>RecipientPickerDialog</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>类</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>收件人选择器(群发):选收件人Excel/TXT并勾选,UI占位</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>(src/GUI/MainGUI.py)[RecipientPickerDialog:1156]</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>2026-08-23 20:37:50</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>onPickFile</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>方法</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>弹文件对话框选xlsx/xls/txt后解析并展示(解析占位)</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>(src/GUI/MainGUI.py)[RecipientPickerDialog-&gt;onPickFile:1230]</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>2026-08-23 20:37:50</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>_loadRecipientsFromFile</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>方法</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>path&lt;str&gt;</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>list&lt;str&gt;</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>从文件读收件人(占位,待接入解析API)</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>(src/GUI/MainGUI.py)[RecipientPickerDialog-&gt;_loadRecipientsFromFile:1244]</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>2026-08-23 20:37:50</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>setRecipients</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>方法</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>recipients&lt;list&lt;str&gt;&gt;</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>用收件人列表填充可勾选列表(默认全选)</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>(src/GUI/MainGUI.py)[RecipientPickerDialog-&gt;setRecipients:1256]</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>2026-08-23 20:37:50</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>_addRecipientItem</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>方法</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>item&lt;QListWidgetItem&gt;</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>把单个收件人条目加入列表</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>(src/GUI/MainGUI.py)[RecipientPickerDialog-&gt;_addRecipientItem:1275]</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>2026-08-23 20:37:50</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>_onItemToggled</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>方法</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>_item</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>列表勾选变化时刷新计数</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>(src/GUI/MainGUI.py)[RecipientPickerDialog-&gt;_onItemToggled:1281]</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>2026-08-23 20:37:50</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>_setAllChecked</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>方法</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>checked&lt;bool&gt;</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>全选或取消全选</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>(src/GUI/MainGUI.py)[RecipientPickerDialog-&gt;_setAllChecked:1285]</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>2026-08-23 20:37:50</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>_checkedRecipients</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>方法</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>list&lt;str&gt;</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>返回当前勾选收件人</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>(src/GUI/MainGUI.py)[RecipientPickerDialog-&gt;_checkedRecipients:1296]</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>2026-08-23 20:37:50</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>getSelectedRecipients</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>方法</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>list&lt;str&gt;</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>供外部读取确定后勾选的收件人</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>(src/GUI/MainGUI.py)[RecipientPickerDialog-&gt;getSelectedRecipients:1304]</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>2026-08-23 20:37:50</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>_updateCount</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>方法</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>刷新已勾选/共计数文案</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>(src/GUI/MainGUI.py)[RecipientPickerDialog-&gt;_updateCount:1312]</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>2026-08-23 20:37:50</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>_updateButtons</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>方法</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>按列表是否为空启用/禁用全选清空按钮</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>(src/GUI/MainGUI.py)[RecipientPickerDialog-&gt;_updateButtons:1318]</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>2026-08-23 20:37:50</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>onPickRecipients</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>方法</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>打开收件人选择器,确定后合并回填收件人框</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>(src/GUI/MainGUI.py)[NormalPage-&gt;onPickRecipients:1592]</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>2026-08-23 20:37:50</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>新增</t>
         </is>
       </c>
     </row>
@@ -8869,7 +9473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9543,7 +10147,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
@@ -9586,7 +10189,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
@@ -9624,7 +10226,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
@@ -9662,6 +10263,408 @@
         </is>
       </c>
       <c r="H24" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>函数名/类名</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>类型</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>参数</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>返回值</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>函数意义</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>位置</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>记录/修改时间</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>isValidEmail</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>函数</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>text&lt;str&gt;</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>判断字符串是否合法邮箱地址</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>(src/activity/recipient_bulk.py)[isValidEmail:21]</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-08-23 20:51:33</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>parseRecipientFile</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>函数</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>path&lt;str&gt;</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>list&lt;str&gt;</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>从Excel(.xlsx/.xls)或TXT读取识别收件人邮箱(去重)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>(src/activity/recipient_bulk.py)[parseRecipientFile:34]</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-08-23 20:51:33</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>_parseTxt</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>函数</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>path&lt;str&gt;</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>list&lt;str&gt;</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>解析TXT逐行识别邮箱</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>(src/activity/recipient_bulk.py)[_parseTxt:58]</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-08-23 20:51:33</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>_parseExcel</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>函数</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>path&lt;str&gt;</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>list&lt;str&gt;</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>按扩展名分发解析Excel</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>(src/activity/recipient_bulk.py)[_parseExcel:72]</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-08-23 20:51:33</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>_parseXlsx</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>函数</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>path&lt;str&gt;</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>list&lt;str&gt;</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>用openpyxl读取xlsx工作表识别邮箱</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>(src/activity/recipient_bulk.py)[_parseXlsx:87]</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-08-23 20:51:33</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>_parseXls</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>函数</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>path&lt;str&gt;</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>list&lt;str&gt;</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>用xlrd读取旧版xls识别邮箱</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>(src/activity/recipient_bulk.py)[_parseXls:105]</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-08-23 20:51:33</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>_dedupKeepOrder</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>函数</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>items&lt;list&lt;str&gt;&gt;</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>list&lt;str&gt;</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>列表去重保持首次顺序</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>(src/activity/recipient_bulk.py)[_dedupKeepOrder:130]</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-08-23 20:51:33</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>mergeRecipients</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>函数</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>current_text&lt;str&gt;; selected&lt;list&lt;str&gt;&gt;</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>合并已有+新增收件人(去重滤空,分号分隔)</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>(src/activity/recipient_bulk.py)[mergeRecipients:143]</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2026-08-23 20:51:33</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>新增</t>
         </is>

</xml_diff>

<commit_message>
build: 新增 macOS 打包支持（.app、CI 工作流、跨平台密钥编译） - PathManager.root() 增加 mac 分支：用户数据放 ~/Library/Application Support/EmailHelper - 新增 邮件助手_mac.spec：BUNDLE 生成 邮件助手.app，扩展取 cred_app*.so - 新增 build_mac.sh：mac 本地一键打包 - 新增 .github/workflows/build-mac.yml：macos-14 CI 自动构建并上传 Release - setup_crypt.py 改为跨平台编译（win=.pyd / mac=.so），复用 cred_app.c 免 Cython
</commit_message>
<xml_diff>
--- a/ProjectDescription/FunctionNameReg.xlsx
+++ b/ProjectDescription/FunctionNameReg.xlsx
@@ -21,6 +21,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="logger" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cred_app" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="store_credentials" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="setup_crypt" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2694,6 +2695,104 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>selectSource</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>函数</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>tuple&lt;str,str&gt;</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>选择扩展源码：优先 .pyx（需 Cython），否则直接用 Cython 产出的 .c</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>(src/security/setup_crypt.py)[selectSource:24]</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>2026-08-25 17:51:05</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>macOS 复用 .c 免装 Cython</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>buildExtensions</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>函数</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>list</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>构建扩展模块列表；.pyx 走 cythonize、.c 直接编译，按平台设置编译参数</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>(src/security/setup_crypt.py)[buildExtensions:35]</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-08-25 17:51:05</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Windows 产 .pyd / macOS 产 .so，保证解密结果一致</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -14930,12 +15029,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-08-23 15:01:25</t>
+          <t>2026-08-25 17:51:05</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>修正开发态=项目根</t>
+          <t>已适配 macOS：打包后用户数据放 ~/Library/Application Support/EmailHelper，Windows 仍为 exe 目录</t>
         </is>
       </c>
     </row>

</xml_diff>